<commit_message>
Fix data consistency: email body and attachment now use same values
- Pre-generate shared variables (trust scale, rate, duration, etc.)
  in each email loop, so body text and attachment content reference
  identical numbers instead of independent random values
- Also add GDP/CPI/PMI data to research_macro_1.pdf attachment,
  consistent with email body
- Regenerate all 100 emails and 90+ attachments with seed 42
- Update DEMO.md with actual values from new data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/attachments/fund_Q1_2024_1.xlsx
+++ b/backend/data/attachments/fund_Q1_2024_1.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.44</v>
+        <v>1.0968</v>
       </c>
       <c r="C2" t="n">
-        <v>1.7558</v>
+        <v>1.2491</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>74514</v>
+        <v>39335</v>
       </c>
     </row>
     <row r="3">
@@ -471,18 +471,18 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.45</v>
+        <v>1.1068</v>
       </c>
       <c r="C3" t="n">
-        <v>1.7658</v>
+        <v>1.2591</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.274</t>
+          <t>0.890</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>74614</v>
+        <v>39435</v>
       </c>
     </row>
     <row r="4">
@@ -492,18 +492,18 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.46</v>
+        <v>1.1168</v>
       </c>
       <c r="C4" t="n">
-        <v>1.7758</v>
+        <v>1.2691</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.971</t>
+          <t>0.382</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>74714</v>
+        <v>39535</v>
       </c>
     </row>
     <row r="5">
@@ -543,12 +543,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CATL</t>
+          <t>Kweichow Moutai</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>China Merchants Bank</t>
+          <t>Ping An</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>